<commit_message>
Re-run Monte Carlo simulation with updated datasets for biogas production
</commit_message>
<xml_diff>
--- a/01_raw_data/Song2023_raw-data.xlsx
+++ b/01_raw_data/Song2023_raw-data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sahar/Documents/methane_letter/01_raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFAFD6A-23C6-1949-8406-EB6D45DEA1D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA98AA8-B636-A443-8AF1-D534F59C6D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1000" yWindow="760" windowWidth="29240" windowHeight="18880" xr2:uid="{DEA953FA-A8F5-E043-B8AF-078D01C0F211}"/>
+    <workbookView xWindow="1020" yWindow="760" windowWidth="29240" windowHeight="18880" xr2:uid="{DEA953FA-A8F5-E043-B8AF-078D01C0F211}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -172,9 +172,6 @@
     <t>flow_m3_per_day</t>
   </si>
   <si>
-    <t>source</t>
-  </si>
-  <si>
     <t>ch4_kg_per_day</t>
   </si>
   <si>
@@ -188,6 +185,9 @@
   </si>
   <si>
     <t>has_ad</t>
+  </si>
+  <si>
+    <t>Song et al Source</t>
   </si>
 </sst>
 </file>
@@ -556,16 +556,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B1" t="s">
         <v>44</v>
       </c>
       <c r="C1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -579,7 +579,7 @@
         <v>56.767123290000001</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -593,7 +593,7 @@
         <v>1853.344077</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -607,7 +607,7 @@
         <v>18694.601129999999</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -621,7 +621,7 @@
         <v>6607.5745370000004</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -635,7 +635,7 @@
         <v>2417.4053180000001</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -649,7 +649,7 @@
         <v>1772.7638999999999</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -663,7 +663,7 @@
         <v>306.2046737</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -677,7 +677,7 @@
         <v>178.4</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -691,7 +691,7 @@
         <v>1521.4285709999999</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -705,7 +705,7 @@
         <v>156</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -719,7 +719,7 @@
         <v>324</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -733,7 +733,7 @@
         <v>194.4</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -747,7 +747,7 @@
         <v>240</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -761,7 +761,7 @@
         <v>295.2</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -775,7 +775,7 @@
         <v>17.48767123</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -789,7 +789,7 @@
         <v>1.8301369860000001</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -803,7 +803,7 @@
         <v>1.35</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -817,7 +817,7 @@
         <v>0.1177</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -831,7 +831,7 @@
         <v>34.5</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -845,7 +845,7 @@
         <v>42.99</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -859,7 +859,7 @@
         <v>56.524999999999999</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -873,7 +873,7 @@
         <v>96.30285714</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -887,7 +887,7 @@
         <v>1.047713E-3</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -901,7 +901,7 @@
         <v>1.794E-3</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -915,7 +915,7 @@
         <v>2.215E-2</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -929,7 +929,7 @@
         <v>21.9</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -943,7 +943,7 @@
         <v>24.5</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -957,7 +957,7 @@
         <v>33</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -971,7 +971,7 @@
         <v>0</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -985,7 +985,7 @@
         <v>21.03905</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
@@ -999,7 +999,7 @@
         <v>286.87</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
@@ -1013,7 +1013,7 @@
         <v>247.07429999999999</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
@@ -1027,7 +1027,7 @@
         <v>0.79650600000000005</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
@@ -1041,7 +1041,7 @@
         <v>3.5267142859999998</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
@@ -1055,7 +1055,7 @@
         <v>3.8879999999999999</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
@@ -1069,7 +1069,7 @@
         <v>22.608000000000001</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -1083,7 +1083,7 @@
         <v>80</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
@@ -1097,7 +1097,7 @@
         <v>105.2054795</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
@@ -1111,7 +1111,7 @@
         <v>46.704599999999999</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
@@ -1125,7 +1125,7 @@
         <v>45.681600000000003</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
@@ -1139,7 +1139,7 @@
         <v>33.814799999999998</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
@@ -1153,7 +1153,7 @@
         <v>53.772599999999997</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
@@ -1167,7 +1167,7 @@
         <v>53.995800000000003</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
@@ -1181,7 +1181,7 @@
         <v>59.724600000000002</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
@@ -1195,7 +1195,7 @@
         <v>86.210999999999999</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
@@ -1209,7 +1209,7 @@
         <v>90.656400000000005</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
@@ -1223,7 +1223,7 @@
         <v>1289.2828360000001</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
@@ -1237,7 +1237,7 @@
         <v>402.90088639999999</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
@@ -1251,7 +1251,7 @@
         <v>1128.122482</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
@@ -1265,7 +1265,7 @@
         <v>5721.1925869999995</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
@@ -1279,7 +1279,7 @@
         <v>12892.82836</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
@@ -1293,7 +1293,7 @@
         <v>1.17</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
@@ -1307,7 +1307,7 @@
         <v>9.63786E-4</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
@@ -1321,7 +1321,7 @@
         <v>3888.24</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
@@ -1335,7 +1335,7 @@
         <v>54.439428569999997</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
@@ -1349,7 +1349,7 @@
         <v>6.9693120000000004</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
@@ -1363,7 +1363,7 @@
         <v>127.52528</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
@@ -1377,7 +1377,7 @@
         <v>2.52E-2</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
@@ -1391,7 +1391,7 @@
         <v>2.8899999999999999E-2</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
@@ -1405,7 +1405,7 @@
         <v>0.50829999999999997</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
@@ -1419,7 +1419,7 @@
         <v>7.3667749999999999E-3</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
@@ -1433,7 +1433,7 @@
         <v>0.497733333</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
@@ -1447,7 +1447,7 @@
         <v>34.200000000000003</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -1461,7 +1461,7 @@
         <v>2880</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -1475,7 +1475,7 @@
         <v>92</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
@@ -1489,7 +1489,7 @@
         <v>161</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
@@ -1503,7 +1503,7 @@
         <v>666.44137799999999</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
@@ -1517,7 +1517,7 @@
         <v>27.40821918</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
@@ -1531,7 +1531,7 @@
         <v>65.106849319999995</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
@@ -1545,7 +1545,7 @@
         <v>208.25753420000001</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -1559,7 +1559,7 @@
         <v>480.04109590000002</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -1573,7 +1573,7 @@
         <v>661.2520548</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
@@ -1587,7 +1587,7 @@
         <v>38.616438359999997</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
@@ -1601,7 +1601,7 @@
         <v>60.802739729999999</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
@@ -1615,7 +1615,7 @@
         <v>1.178082192</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
@@ -1629,7 +1629,7 @@
         <v>376.74546700000002</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
@@ -1643,7 +1643,7 @@
         <v>0.26400000000000001</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
@@ -1657,7 +1657,7 @@
         <v>0.45329999999999998</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -1671,7 +1671,7 @@
         <v>618.72006599999997</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
@@ -1685,7 +1685,7 @@
         <v>1271.2328769999999</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
@@ -1699,7 +1699,7 @@
         <v>0.157466667</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
@@ -1713,7 +1713,7 @@
         <v>84</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
@@ -1727,7 +1727,7 @@
         <v>87.408219180000003</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
@@ -1741,7 +1741,7 @@
         <v>221.61369859999999</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
@@ -1755,7 +1755,7 @@
         <v>2476.8000000000002</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
@@ -1769,7 +1769,7 @@
         <v>744</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -1783,7 +1783,7 @@
         <v>4896</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
@@ -1797,7 +1797,7 @@
         <v>6960</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -1811,7 +1811,7 @@
         <v>10248</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -1825,7 +1825,7 @@
         <v>1968</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
@@ -1839,7 +1839,7 @@
         <v>2184</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
@@ -1853,7 +1853,7 @@
         <v>1992</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
@@ -1867,7 +1867,7 @@
         <v>3120</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
@@ -1881,7 +1881,7 @@
         <v>5496</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
@@ -1895,7 +1895,7 @@
         <v>1488</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
@@ -1909,7 +1909,7 @@
         <v>1920</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
@@ -1923,7 +1923,7 @@
         <v>302</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
@@ -1937,7 +1937,7 @@
         <v>247.67123290000001</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
@@ -1951,7 +1951,7 @@
         <v>285</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
@@ -1965,7 +1965,7 @@
         <v>206.4</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
@@ -1979,7 +1979,7 @@
         <v>69.599999999999994</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
@@ -1993,7 +1993,7 @@
         <v>340</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
@@ -2007,7 +2007,7 @@
         <v>65.599999999999994</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.2">
@@ -2021,7 +2021,7 @@
         <v>624.48</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
@@ -2035,7 +2035,7 @@
         <v>1644.48</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
@@ -2049,7 +2049,7 @@
         <v>2214.2399999999998</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -2063,7 +2063,7 @@
         <v>2026.08</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
@@ -2077,7 +2077,7 @@
         <v>760.8</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
@@ -2091,7 +2091,7 @@
         <v>253.2</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
@@ -2105,7 +2105,7 @@
         <v>119.76</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
@@ -2119,7 +2119,7 @@
         <v>164.16</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
@@ -2133,7 +2133,7 @@
         <v>941.28</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>